<commit_message>
feat: derive attendance status (LEAVE/HOLIDAY/WEEKEND) + readable adjustment history
</commit_message>
<xml_diff>
--- a/attendance_demo_HR_2026_06_chinh_lai.xlsx
+++ b/attendance_demo_HR_2026_06_chinh_lai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EE74AA-4D61-4AA6-964C-B8D9AF08819A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E7519D-4845-4962-9C52-B56219ECB9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="17">
   <si>
     <t>employeeCode</t>
   </si>
@@ -37,12 +37,6 @@
     <t>timeOut</t>
   </si>
   <si>
-    <t>attendanceStatus</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
     <t>EMP004</t>
   </si>
   <si>
@@ -61,34 +55,22 @@
     <t>17:00</t>
   </si>
   <si>
-    <t>PRESENT</t>
-  </si>
-  <si>
     <t>2026-06-02</t>
   </si>
   <si>
     <t>08:10</t>
   </si>
   <si>
-    <t>LATE</t>
-  </si>
-  <si>
-    <t>Kẹt xe</t>
-  </si>
-  <si>
     <t>EMP005</t>
   </si>
   <si>
     <t>Vũ Thị Nhân Sự</t>
   </si>
   <si>
-    <t>ABSENT</t>
-  </si>
-  <si>
-    <t>Nghỉ phép năm</t>
-  </si>
-  <si>
     <t>Department</t>
+  </si>
+  <si>
+    <t>2026-06-19</t>
   </si>
 </sst>
 </file>
@@ -151,59 +133,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF4C1130"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFEADCF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -221,16 +161,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{ABDCFF9C-E678-479E-B4CF-266188AD75D7}" name="Attendance_HR_Table33" displayName="Attendance_HR_Table33" ref="A1:H5">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{ABDCFF9C-E678-479E-B4CF-266188AD75D7}" name="Attendance_HR_Table33" displayName="Attendance_HR_Table33" ref="A1:F6">
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6BC99C56-54B7-4D23-80D1-90EF04757EAF}" name="employeeCode"/>
     <tableColumn id="7" xr3:uid="{27AABD0D-3063-4FFB-A9B2-817FA36F656E}" name="fullName"/>
     <tableColumn id="8" xr3:uid="{C7A53E08-B37F-47A2-B882-D94B40FC1622}" name="Department"/>
     <tableColumn id="2" xr3:uid="{4E1456A0-64C0-48C0-9734-1C94AC89C87D}" name="workDate"/>
-    <tableColumn id="3" xr3:uid="{A6DBBFE5-ED59-43B9-BF22-74602E59715B}" name="timeIn" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{A6DBBFE5-ED59-43B9-BF22-74602E59715B}" name="timeIn" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{6DBCF681-0CE4-4A7B-9C6A-BCF74D627578}" name="timeOut"/>
-    <tableColumn id="5" xr3:uid="{93825079-1A99-49E2-882F-9F6D0A0C195B}" name="attendanceStatus"/>
-    <tableColumn id="6" xr3:uid="{DF353C0C-1468-46D3-AA48-E98DF566FC84}" name="note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -521,19 +459,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="20.5546875" customWidth="1"/>
     <col min="4" max="4" width="18.77734375" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="4"/>
-    <col min="7" max="7" width="18.6640625" customWidth="1"/>
-    <col min="8" max="8" width="17.88671875" customWidth="1"/>
+    <col min="5" max="5" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -541,7 +477,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -552,128 +488,100 @@
       <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="5">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="3" t="s">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" t="s">
-        <v>21</v>
-      </c>
+      <c r="E6" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G5">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>G2="PRESENT"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>G2="LATE"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>G2="ABSENT"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>G2="UNEXCUSED"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="G2:G5" xr:uid="{74CC875A-DF32-496B-AFC1-CFA0AFEAD680}">
-      <formula1>"PRESENT,LATE,ABSENT,UNEXCUSED"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Add validate for attendance and change status in case employee is absent when having the leaving form
</commit_message>
<xml_diff>
--- a/attendance_demo_HR_2026_06_chinh_lai.xlsx
+++ b/attendance_demo_HR_2026_06_chinh_lai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EE74AA-4D61-4AA6-964C-B8D9AF08819A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06592C8B-D33C-4E6D-95E0-675169200281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="17">
   <si>
     <t>employeeCode</t>
   </si>
@@ -37,12 +37,6 @@
     <t>timeOut</t>
   </si>
   <si>
-    <t>attendanceStatus</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
     <t>EMP004</t>
   </si>
   <si>
@@ -61,34 +55,22 @@
     <t>17:00</t>
   </si>
   <si>
-    <t>PRESENT</t>
-  </si>
-  <si>
     <t>2026-06-02</t>
   </si>
   <si>
     <t>08:10</t>
   </si>
   <si>
-    <t>LATE</t>
-  </si>
-  <si>
-    <t>Kẹt xe</t>
-  </si>
-  <si>
     <t>EMP005</t>
   </si>
   <si>
     <t>Vũ Thị Nhân Sự</t>
   </si>
   <si>
-    <t>ABSENT</t>
-  </si>
-  <si>
-    <t>Nghỉ phép năm</t>
-  </si>
-  <si>
     <t>Department</t>
+  </si>
+  <si>
+    <t>2026-06-19</t>
   </si>
 </sst>
 </file>
@@ -151,59 +133,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF4C1130"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFEADCF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -221,16 +161,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{ABDCFF9C-E678-479E-B4CF-266188AD75D7}" name="Attendance_HR_Table33" displayName="Attendance_HR_Table33" ref="A1:H5">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{ABDCFF9C-E678-479E-B4CF-266188AD75D7}" name="Attendance_HR_Table33" displayName="Attendance_HR_Table33" ref="A1:F5">
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6BC99C56-54B7-4D23-80D1-90EF04757EAF}" name="employeeCode"/>
     <tableColumn id="7" xr3:uid="{27AABD0D-3063-4FFB-A9B2-817FA36F656E}" name="fullName"/>
     <tableColumn id="8" xr3:uid="{C7A53E08-B37F-47A2-B882-D94B40FC1622}" name="Department"/>
     <tableColumn id="2" xr3:uid="{4E1456A0-64C0-48C0-9734-1C94AC89C87D}" name="workDate"/>
-    <tableColumn id="3" xr3:uid="{A6DBBFE5-ED59-43B9-BF22-74602E59715B}" name="timeIn" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{A6DBBFE5-ED59-43B9-BF22-74602E59715B}" name="timeIn" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{6DBCF681-0CE4-4A7B-9C6A-BCF74D627578}" name="timeOut"/>
-    <tableColumn id="5" xr3:uid="{93825079-1A99-49E2-882F-9F6D0A0C195B}" name="attendanceStatus"/>
-    <tableColumn id="6" xr3:uid="{DF353C0C-1468-46D3-AA48-E98DF566FC84}" name="note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -521,19 +459,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="20.5546875" customWidth="1"/>
     <col min="4" max="4" width="18.77734375" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="4"/>
+    <col min="5" max="5" width="8.88671875" style="3"/>
     <col min="7" max="7" width="18.6640625" customWidth="1"/>
     <col min="8" max="8" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -541,7 +479,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -552,128 +490,99 @@
       <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="5">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="3" t="s">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="H3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G5">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>G2="PRESENT"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>G2="LATE"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>G2="ABSENT"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>G2="UNEXCUSED"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="G2:G5" xr:uid="{74CC875A-DF32-496B-AFC1-CFA0AFEAD680}">
-      <formula1>"PRESENT,LATE,ABSENT,UNEXCUSED"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>